<commit_message>
Publish reorder snapshots (Miami 05.26.26, China 05.26.26)
</commit_message>
<xml_diff>
--- a/china-dashboard/public/data/latest.xlsx
+++ b/china-dashboard/public/data/latest.xlsx
@@ -426,7 +426,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:P42"/>
+  <dimension ref="A1:P44"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -579,7 +579,7 @@
         <v>0</v>
       </c>
       <c r="M2" t="n">
-        <v>2.94</v>
+        <v>2.91</v>
       </c>
       <c r="N2" t="n">
         <v>78</v>
@@ -588,7 +588,7 @@
         <v>1</v>
       </c>
       <c r="P2" t="n">
-        <v>20</v>
+        <v>10</v>
       </c>
     </row>
     <row r="3">
@@ -623,19 +623,19 @@
         </is>
       </c>
       <c r="G3" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="H3" t="n">
         <v>40</v>
       </c>
       <c r="I3" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J3" t="n">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="K3" t="n">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="L3" t="b">
         <v>0</v>
@@ -691,7 +691,7 @@
         <v>20</v>
       </c>
       <c r="I4" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="J4" t="n">
         <v>49</v>
@@ -703,7 +703,7 @@
         <v>0</v>
       </c>
       <c r="M4" t="n">
-        <v>0.71</v>
+        <v>0.75</v>
       </c>
       <c r="N4" t="n">
         <v>23</v>
@@ -747,25 +747,25 @@
         </is>
       </c>
       <c r="G5" t="n">
-        <v>19</v>
+        <v>17</v>
       </c>
       <c r="H5" t="n">
         <v>20</v>
       </c>
       <c r="I5" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="J5" t="n">
-        <v>42</v>
+        <v>40</v>
       </c>
       <c r="K5" t="n">
-        <v>42</v>
+        <v>40</v>
       </c>
       <c r="L5" t="b">
         <v>0</v>
       </c>
       <c r="M5" t="n">
-        <v>0.97</v>
+        <v>0.92</v>
       </c>
       <c r="N5" t="n">
         <v>23</v>
@@ -815,7 +815,7 @@
         <v>61</v>
       </c>
       <c r="I6" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="J6" t="n">
         <v>61</v>
@@ -933,7 +933,7 @@
         </is>
       </c>
       <c r="G8" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="H8" t="n">
         <v>40</v>
@@ -942,16 +942,16 @@
         <v>1</v>
       </c>
       <c r="J8" t="n">
-        <v>47</v>
+        <v>45</v>
       </c>
       <c r="K8" t="n">
-        <v>47</v>
+        <v>45</v>
       </c>
       <c r="L8" t="b">
         <v>0</v>
       </c>
       <c r="M8" t="n">
-        <v>1.1</v>
+        <v>1.12</v>
       </c>
       <c r="N8" t="n">
         <v>30</v>
@@ -995,25 +995,25 @@
         </is>
       </c>
       <c r="G9" t="n">
-        <v>45</v>
+        <v>42</v>
       </c>
       <c r="H9" t="n">
         <v>201</v>
       </c>
       <c r="I9" t="n">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="J9" t="n">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="K9" t="n">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="L9" t="b">
         <v>0</v>
       </c>
       <c r="M9" t="n">
-        <v>5.61</v>
+        <v>5.54</v>
       </c>
       <c r="N9" t="n">
         <v>148</v>
@@ -1057,25 +1057,25 @@
         </is>
       </c>
       <c r="G10" t="n">
-        <v>42</v>
+        <v>40</v>
       </c>
       <c r="H10" t="n">
         <v>60</v>
       </c>
       <c r="I10" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="J10" t="n">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="K10" t="n">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="L10" t="b">
         <v>0</v>
       </c>
       <c r="M10" t="n">
-        <v>2.04</v>
+        <v>2</v>
       </c>
       <c r="N10" t="n">
         <v>51</v>
@@ -1119,25 +1119,25 @@
         </is>
       </c>
       <c r="G11" t="n">
-        <v>26</v>
+        <v>24</v>
       </c>
       <c r="H11" t="n">
         <v>20</v>
       </c>
       <c r="I11" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J11" t="n">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="K11" t="n">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="L11" t="b">
         <v>0</v>
       </c>
       <c r="M11" t="n">
-        <v>1.1</v>
+        <v>1.13</v>
       </c>
       <c r="N11" t="n">
         <v>27</v>
@@ -1181,13 +1181,13 @@
         </is>
       </c>
       <c r="G12" t="n">
-        <v>165</v>
+        <v>162</v>
       </c>
       <c r="H12" t="n">
         <v>160</v>
       </c>
       <c r="I12" t="n">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="J12" t="n">
         <v>55</v>
@@ -1199,7 +1199,7 @@
         <v>0</v>
       </c>
       <c r="M12" t="n">
-        <v>6.29</v>
+        <v>6.44</v>
       </c>
       <c r="N12" t="n">
         <v>155</v>
@@ -1243,25 +1243,25 @@
         </is>
       </c>
       <c r="G13" t="n">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="H13" t="n">
         <v>140</v>
       </c>
       <c r="I13" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="J13" t="n">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="K13" t="n">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="L13" t="b">
         <v>0</v>
       </c>
       <c r="M13" t="n">
-        <v>2.61</v>
+        <v>2.53</v>
       </c>
       <c r="N13" t="n">
         <v>49</v>
@@ -1323,7 +1323,7 @@
         <v>0</v>
       </c>
       <c r="M14" t="n">
-        <v>0.91</v>
+        <v>0.89</v>
       </c>
       <c r="N14" t="n">
         <v>25</v>
@@ -1385,7 +1385,7 @@
         <v>1</v>
       </c>
       <c r="M15" t="n">
-        <v>4.17</v>
+        <v>4.03</v>
       </c>
       <c r="N15" t="n">
         <v>123</v>
@@ -1394,7 +1394,7 @@
         <v>1</v>
       </c>
       <c r="P15" t="n">
-        <v>130</v>
+        <v>120</v>
       </c>
     </row>
     <row r="16">
@@ -1497,7 +1497,7 @@
         <v>20</v>
       </c>
       <c r="I17" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="J17" t="n">
         <v>1</v>
@@ -1509,7 +1509,7 @@
         <v>0</v>
       </c>
       <c r="M17" t="n">
-        <v>0.71</v>
+        <v>0.74</v>
       </c>
       <c r="N17" t="n">
         <v>15</v>
@@ -1518,7 +1518,7 @@
         <v>1</v>
       </c>
       <c r="P17" t="n">
-        <v>20</v>
+        <v>30</v>
       </c>
     </row>
     <row r="18">
@@ -1553,25 +1553,25 @@
         </is>
       </c>
       <c r="G18" t="n">
-        <v>898</v>
+        <v>893</v>
       </c>
       <c r="H18" t="n">
         <v>1000</v>
       </c>
       <c r="I18" t="n">
-        <v>57</v>
+        <v>55</v>
       </c>
       <c r="J18" t="n">
-        <v>64</v>
+        <v>63</v>
       </c>
       <c r="K18" t="n">
-        <v>64</v>
+        <v>63</v>
       </c>
       <c r="L18" t="b">
         <v>0</v>
       </c>
       <c r="M18" t="n">
-        <v>33.05</v>
+        <v>32.87</v>
       </c>
       <c r="N18" t="n">
         <v>924</v>
@@ -1615,25 +1615,25 @@
         </is>
       </c>
       <c r="G19" t="n">
-        <v>1378</v>
+        <v>1362</v>
       </c>
       <c r="H19" t="n">
         <v>5</v>
       </c>
       <c r="I19" t="n">
-        <v>93</v>
+        <v>102</v>
       </c>
       <c r="J19" t="n">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="K19" t="n">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="L19" t="b">
         <v>0</v>
       </c>
       <c r="M19" t="n">
-        <v>27.16</v>
+        <v>26.93</v>
       </c>
       <c r="N19" t="n">
         <v>765</v>
@@ -1642,7 +1642,7 @@
         <v>1</v>
       </c>
       <c r="P19" t="n">
-        <v>160</v>
+        <v>150</v>
       </c>
     </row>
     <row r="20">
@@ -1677,13 +1677,13 @@
         </is>
       </c>
       <c r="G20" t="n">
-        <v>122</v>
+        <v>121</v>
       </c>
       <c r="H20" t="n">
         <v>0</v>
       </c>
       <c r="I20" t="n">
-        <v>10</v>
+        <v>8</v>
       </c>
       <c r="J20" t="n">
         <v>48</v>
@@ -1695,7 +1695,7 @@
         <v>0</v>
       </c>
       <c r="M20" t="n">
-        <v>2.86</v>
+        <v>2.84</v>
       </c>
       <c r="N20" t="n">
         <v>81</v>
@@ -1704,7 +1704,7 @@
         <v>1</v>
       </c>
       <c r="P20" t="n">
-        <v>40</v>
+        <v>50</v>
       </c>
     </row>
     <row r="21">
@@ -1745,7 +1745,7 @@
         <v>0</v>
       </c>
       <c r="I21" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="J21" t="n">
         <v>58</v>
@@ -1757,7 +1757,7 @@
         <v>0</v>
       </c>
       <c r="M21" t="n">
-        <v>1.14</v>
+        <v>1.1</v>
       </c>
       <c r="N21" t="n">
         <v>28</v>
@@ -1819,7 +1819,7 @@
         <v>1</v>
       </c>
       <c r="M22" t="n">
-        <v>0.5</v>
+        <v>0.48</v>
       </c>
       <c r="N22" t="n">
         <v>16</v>
@@ -1881,7 +1881,7 @@
         <v>0</v>
       </c>
       <c r="M23" t="n">
-        <v>4.15</v>
+        <v>4.1</v>
       </c>
       <c r="N23" t="n">
         <v>135</v>
@@ -1890,7 +1890,7 @@
         <v>1</v>
       </c>
       <c r="P23" t="n">
-        <v>50</v>
+        <v>40</v>
       </c>
     </row>
     <row r="24">
@@ -1901,17 +1901,17 @@
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>BR4238</t>
+          <t>KT8100</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>BR4238_FBA</t>
+          <t>KT8100_FBA</t>
         </is>
       </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t>B0B78BR6NM</t>
+          <t>B0742QYGGN</t>
         </is>
       </c>
       <c r="E24" t="inlineStr">
@@ -1925,28 +1925,28 @@
         </is>
       </c>
       <c r="G24" t="n">
-        <v>15</v>
+        <v>158</v>
       </c>
       <c r="H24" t="n">
-        <v>0</v>
+        <v>60</v>
       </c>
       <c r="I24" t="n">
-        <v>0</v>
+        <v>7</v>
       </c>
       <c r="J24" t="n">
-        <v>44</v>
+        <v>57</v>
       </c>
       <c r="K24" t="n">
-        <v>44</v>
+        <v>57</v>
       </c>
       <c r="L24" t="b">
         <v>0</v>
       </c>
       <c r="M24" t="n">
-        <v>0.37</v>
+        <v>3.77</v>
       </c>
       <c r="N24" t="n">
-        <v>10</v>
+        <v>111</v>
       </c>
       <c r="O24" t="b">
         <v>1</v>
@@ -1958,125 +1958,125 @@
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>NC CHOKERS</t>
+          <t>PJ + FJ JEWELRY</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>NC4297</t>
+          <t>BR4238</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>NC4297_FBA</t>
+          <t>BR4238_FBA</t>
         </is>
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t>B09826V9Z8</t>
+          <t>B0B78BR6NM</t>
         </is>
       </c>
       <c r="E25" t="inlineStr">
         <is>
-          <t>NC4285-Master</t>
+          <t>KT8100-Master</t>
         </is>
       </c>
       <c r="F25" t="inlineStr">
         <is>
-          <t>NC</t>
+          <t>PJ</t>
         </is>
       </c>
       <c r="G25" t="n">
-        <v>331</v>
+        <v>15</v>
       </c>
       <c r="H25" t="n">
-        <v>3600</v>
+        <v>0</v>
       </c>
       <c r="I25" t="n">
-        <v>82</v>
+        <v>0</v>
       </c>
       <c r="J25" t="n">
-        <v>0</v>
+        <v>44</v>
       </c>
       <c r="K25" t="n">
-        <v>4.6</v>
+        <v>44</v>
       </c>
       <c r="L25" t="b">
         <v>0</v>
       </c>
       <c r="M25" t="n">
-        <v>72.5</v>
+        <v>0.34</v>
       </c>
       <c r="N25" t="n">
-        <v>2066</v>
+        <v>10</v>
       </c>
       <c r="O25" t="b">
         <v>1</v>
       </c>
       <c r="P25" t="n">
-        <v>340</v>
+        <v>10</v>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>NC CHOKERS</t>
+          <t>PJ + FJ JEWELRY</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>NC4367</t>
+          <t>BN1663</t>
         </is>
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>NC4367_FBA</t>
+          <t>BN1663_FBA</t>
         </is>
       </c>
       <c r="D26" t="inlineStr">
         <is>
-          <t>B0BZB723JD</t>
+          <t>B072PX13TJ</t>
         </is>
       </c>
       <c r="E26" t="inlineStr">
         <is>
-          <t>NC4285-Master</t>
+          <t>BN1663-Master</t>
         </is>
       </c>
       <c r="F26" t="inlineStr">
         <is>
-          <t>NC</t>
+          <t>PJ</t>
         </is>
       </c>
       <c r="G26" t="n">
-        <v>570</v>
+        <v>29</v>
       </c>
       <c r="H26" t="n">
-        <v>120</v>
+        <v>41</v>
       </c>
       <c r="I26" t="n">
-        <v>16</v>
+        <v>2</v>
       </c>
       <c r="J26" t="n">
-        <v>57</v>
+        <v>55</v>
       </c>
       <c r="K26" t="n">
-        <v>57</v>
+        <v>55</v>
       </c>
       <c r="L26" t="b">
         <v>0</v>
       </c>
       <c r="M26" t="n">
-        <v>13.68</v>
+        <v>1.2</v>
       </c>
       <c r="N26" t="n">
-        <v>371</v>
+        <v>32</v>
       </c>
       <c r="O26" t="b">
         <v>1</v>
       </c>
       <c r="P26" t="n">
-        <v>120</v>
+        <v>10</v>
       </c>
     </row>
     <row r="27">
@@ -2087,17 +2087,17 @@
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>NC4290-1</t>
+          <t>NC4297</t>
         </is>
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>NC4290-1</t>
+          <t>NC4297_FBA</t>
         </is>
       </c>
       <c r="D27" t="inlineStr">
         <is>
-          <t>B0DGWDSSKW</t>
+          <t>B09826V9Z8</t>
         </is>
       </c>
       <c r="E27" t="inlineStr">
@@ -2111,34 +2111,34 @@
         </is>
       </c>
       <c r="G27" t="n">
-        <v>82</v>
+        <v>330</v>
       </c>
       <c r="H27" t="n">
-        <v>480</v>
+        <v>3600</v>
       </c>
       <c r="I27" t="n">
-        <v>4</v>
+        <v>88</v>
       </c>
       <c r="J27" t="n">
-        <v>58</v>
+        <v>0</v>
       </c>
       <c r="K27" t="n">
-        <v>58</v>
+        <v>4.6</v>
       </c>
       <c r="L27" t="b">
         <v>0</v>
       </c>
       <c r="M27" t="n">
-        <v>10.91</v>
+        <v>71.47</v>
       </c>
       <c r="N27" t="n">
-        <v>283</v>
+        <v>2066</v>
       </c>
       <c r="O27" t="b">
         <v>1</v>
       </c>
       <c r="P27" t="n">
-        <v>90</v>
+        <v>270</v>
       </c>
     </row>
     <row r="28">
@@ -2149,17 +2149,17 @@
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>NC4303</t>
+          <t>NC4367</t>
         </is>
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>NC4303_FBA</t>
+          <t>NC4367_FBA</t>
         </is>
       </c>
       <c r="D28" t="inlineStr">
         <is>
-          <t>B09825SRFQ</t>
+          <t>B0BZB723JD</t>
         </is>
       </c>
       <c r="E28" t="inlineStr">
@@ -2173,34 +2173,34 @@
         </is>
       </c>
       <c r="G28" t="n">
-        <v>185</v>
+        <v>561</v>
       </c>
       <c r="H28" t="n">
-        <v>60</v>
+        <v>120</v>
       </c>
       <c r="I28" t="n">
-        <v>5</v>
+        <v>23</v>
       </c>
       <c r="J28" t="n">
-        <v>47</v>
+        <v>56</v>
       </c>
       <c r="K28" t="n">
-        <v>47</v>
+        <v>56</v>
       </c>
       <c r="L28" t="b">
         <v>0</v>
       </c>
       <c r="M28" t="n">
-        <v>5.14</v>
+        <v>13.4</v>
       </c>
       <c r="N28" t="n">
-        <v>164</v>
+        <v>371</v>
       </c>
       <c r="O28" t="b">
         <v>1</v>
       </c>
       <c r="P28" t="n">
-        <v>60</v>
+        <v>100</v>
       </c>
     </row>
     <row r="29">
@@ -2211,17 +2211,17 @@
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>NC4342</t>
+          <t>NC4290-1</t>
         </is>
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>NC4342_FBA</t>
+          <t>NC4290-1</t>
         </is>
       </c>
       <c r="D29" t="inlineStr">
         <is>
-          <t>B0B73XGZSM</t>
+          <t>B0DGWDSSKW</t>
         </is>
       </c>
       <c r="E29" t="inlineStr">
@@ -2235,34 +2235,34 @@
         </is>
       </c>
       <c r="G29" t="n">
-        <v>19</v>
+        <v>76</v>
       </c>
       <c r="H29" t="n">
-        <v>80</v>
+        <v>475</v>
       </c>
       <c r="I29" t="n">
-        <v>0</v>
+        <v>8</v>
       </c>
       <c r="J29" t="n">
-        <v>78</v>
+        <v>58</v>
       </c>
       <c r="K29" t="n">
-        <v>78</v>
+        <v>58</v>
       </c>
       <c r="L29" t="b">
         <v>0</v>
       </c>
       <c r="M29" t="n">
-        <v>1.76</v>
+        <v>10.91</v>
       </c>
       <c r="N29" t="n">
-        <v>44</v>
+        <v>283</v>
       </c>
       <c r="O29" t="b">
         <v>1</v>
       </c>
       <c r="P29" t="n">
-        <v>10</v>
+        <v>100</v>
       </c>
     </row>
     <row r="30">
@@ -2273,22 +2273,22 @@
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>NC4270</t>
+          <t>NC4303</t>
         </is>
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>NC4270_FBA</t>
+          <t>NC4303_FBA</t>
         </is>
       </c>
       <c r="D30" t="inlineStr">
         <is>
-          <t>B082LRFT53</t>
+          <t>B09825SRFQ</t>
         </is>
       </c>
       <c r="E30" t="inlineStr">
         <is>
-          <t>NC4058-Master</t>
+          <t>NC4285-Master</t>
         </is>
       </c>
       <c r="F30" t="inlineStr">
@@ -2297,34 +2297,34 @@
         </is>
       </c>
       <c r="G30" t="n">
-        <v>22</v>
+        <v>183</v>
       </c>
       <c r="H30" t="n">
-        <v>80</v>
+        <v>60</v>
       </c>
       <c r="I30" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="J30" t="n">
-        <v>61</v>
+        <v>47</v>
       </c>
       <c r="K30" t="n">
-        <v>61</v>
+        <v>47</v>
       </c>
       <c r="L30" t="b">
         <v>0</v>
       </c>
       <c r="M30" t="n">
-        <v>1.98</v>
+        <v>5.25</v>
       </c>
       <c r="N30" t="n">
-        <v>56</v>
+        <v>164</v>
       </c>
       <c r="O30" t="b">
         <v>1</v>
       </c>
       <c r="P30" t="n">
-        <v>20</v>
+        <v>70</v>
       </c>
     </row>
     <row r="31">
@@ -2335,22 +2335,22 @@
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>NC4273</t>
+          <t>NC4342</t>
         </is>
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>NC4273_FBA</t>
+          <t>NC4342_FBA</t>
         </is>
       </c>
       <c r="D31" t="inlineStr">
         <is>
-          <t>B082LMC563</t>
+          <t>B0B73XGZSM</t>
         </is>
       </c>
       <c r="E31" t="inlineStr">
         <is>
-          <t>NC4058-Master</t>
+          <t>NC4285-Master</t>
         </is>
       </c>
       <c r="F31" t="inlineStr">
@@ -2359,34 +2359,34 @@
         </is>
       </c>
       <c r="G31" t="n">
-        <v>46</v>
+        <v>20</v>
       </c>
       <c r="H31" t="n">
-        <v>0</v>
+        <v>80</v>
       </c>
       <c r="I31" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="J31" t="n">
-        <v>29</v>
+        <v>78</v>
       </c>
       <c r="K31" t="n">
-        <v>29</v>
+        <v>78</v>
       </c>
       <c r="L31" t="b">
         <v>0</v>
       </c>
       <c r="M31" t="n">
-        <v>1.32</v>
+        <v>1.79</v>
       </c>
       <c r="N31" t="n">
-        <v>39</v>
+        <v>44</v>
       </c>
       <c r="O31" t="b">
         <v>1</v>
       </c>
       <c r="P31" t="n">
-        <v>40</v>
+        <v>10</v>
       </c>
     </row>
     <row r="32">
@@ -2397,22 +2397,22 @@
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>NC4059-1</t>
+          <t>NC4270</t>
         </is>
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>NC4059-1</t>
+          <t>NC4270_FBA</t>
         </is>
       </c>
       <c r="D32" t="inlineStr">
         <is>
-          <t>B0DDT2L7FL</t>
+          <t>B082LRFT53</t>
         </is>
       </c>
       <c r="E32" t="inlineStr">
         <is>
-          <t>NC4059-Master</t>
+          <t>NC4058-Master</t>
         </is>
       </c>
       <c r="F32" t="inlineStr">
@@ -2421,34 +2421,34 @@
         </is>
       </c>
       <c r="G32" t="n">
-        <v>88</v>
+        <v>19</v>
       </c>
       <c r="H32" t="n">
-        <v>401</v>
+        <v>80</v>
       </c>
       <c r="I32" t="n">
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="J32" t="n">
-        <v>67</v>
+        <v>59</v>
       </c>
       <c r="K32" t="n">
-        <v>67</v>
+        <v>59</v>
       </c>
       <c r="L32" t="b">
         <v>0</v>
       </c>
       <c r="M32" t="n">
-        <v>9.51</v>
+        <v>2.08</v>
       </c>
       <c r="N32" t="n">
-        <v>211</v>
+        <v>56</v>
       </c>
       <c r="O32" t="b">
         <v>1</v>
       </c>
       <c r="P32" t="n">
-        <v>80</v>
+        <v>20</v>
       </c>
     </row>
     <row r="33">
@@ -2459,22 +2459,22 @@
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>NC4084-1</t>
+          <t>NC4273</t>
         </is>
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>NC4084-1_FBA</t>
+          <t>NC4273_FBA</t>
         </is>
       </c>
       <c r="D33" t="inlineStr">
         <is>
-          <t>B07WNRW3SV</t>
+          <t>B082LMC563</t>
         </is>
       </c>
       <c r="E33" t="inlineStr">
         <is>
-          <t>NC4059-Master</t>
+          <t>NC4058-Master</t>
         </is>
       </c>
       <c r="F33" t="inlineStr">
@@ -2483,34 +2483,34 @@
         </is>
       </c>
       <c r="G33" t="n">
-        <v>194</v>
+        <v>46</v>
       </c>
       <c r="H33" t="n">
+        <v>0</v>
+      </c>
+      <c r="I33" t="n">
+        <v>2</v>
+      </c>
+      <c r="J33" t="n">
+        <v>29</v>
+      </c>
+      <c r="K33" t="n">
+        <v>29</v>
+      </c>
+      <c r="L33" t="b">
+        <v>0</v>
+      </c>
+      <c r="M33" t="n">
+        <v>1.26</v>
+      </c>
+      <c r="N33" t="n">
+        <v>39</v>
+      </c>
+      <c r="O33" t="b">
+        <v>1</v>
+      </c>
+      <c r="P33" t="n">
         <v>30</v>
-      </c>
-      <c r="I33" t="n">
-        <v>7</v>
-      </c>
-      <c r="J33" t="n">
-        <v>44</v>
-      </c>
-      <c r="K33" t="n">
-        <v>44</v>
-      </c>
-      <c r="L33" t="b">
-        <v>0</v>
-      </c>
-      <c r="M33" t="n">
-        <v>5.02</v>
-      </c>
-      <c r="N33" t="n">
-        <v>115</v>
-      </c>
-      <c r="O33" t="b">
-        <v>1</v>
-      </c>
-      <c r="P33" t="n">
-        <v>80</v>
       </c>
     </row>
     <row r="34">
@@ -2521,17 +2521,17 @@
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>NC4284</t>
+          <t>NC4059-1</t>
         </is>
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>NC4284_FBA</t>
+          <t>NC4059-1</t>
         </is>
       </c>
       <c r="D34" t="inlineStr">
         <is>
-          <t>B08Q31XC28</t>
+          <t>B0DDT2L7FL</t>
         </is>
       </c>
       <c r="E34" t="inlineStr">
@@ -2545,34 +2545,34 @@
         </is>
       </c>
       <c r="G34" t="n">
-        <v>5</v>
+        <v>87</v>
       </c>
       <c r="H34" t="n">
-        <v>80</v>
+        <v>401</v>
       </c>
       <c r="I34" t="n">
-        <v>0</v>
+        <v>13</v>
       </c>
       <c r="J34" t="n">
-        <v>55</v>
+        <v>66</v>
       </c>
       <c r="K34" t="n">
-        <v>55</v>
+        <v>66</v>
       </c>
       <c r="L34" t="b">
         <v>0</v>
       </c>
       <c r="M34" t="n">
-        <v>1.91</v>
+        <v>9.300000000000001</v>
       </c>
       <c r="N34" t="n">
-        <v>53</v>
+        <v>211</v>
       </c>
       <c r="O34" t="b">
         <v>1</v>
       </c>
       <c r="P34" t="n">
-        <v>30</v>
+        <v>60</v>
       </c>
     </row>
     <row r="35">
@@ -2583,17 +2583,17 @@
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>NC4059</t>
+          <t>NC4084-1</t>
         </is>
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>NC4059_FBA</t>
+          <t>NC4084-1_FBA</t>
         </is>
       </c>
       <c r="D35" t="inlineStr">
         <is>
-          <t>B01IACWDOK</t>
+          <t>B07WNRW3SV</t>
         </is>
       </c>
       <c r="E35" t="inlineStr">
@@ -2607,34 +2607,34 @@
         </is>
       </c>
       <c r="G35" t="n">
-        <v>21</v>
+        <v>188</v>
       </c>
       <c r="H35" t="n">
-        <v>87</v>
+        <v>30</v>
       </c>
       <c r="I35" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="J35" t="n">
-        <v>41</v>
+        <v>43</v>
       </c>
       <c r="K35" t="n">
-        <v>41</v>
+        <v>43</v>
       </c>
       <c r="L35" t="b">
         <v>0</v>
       </c>
       <c r="M35" t="n">
-        <v>2.6</v>
+        <v>4.95</v>
       </c>
       <c r="N35" t="n">
-        <v>79</v>
+        <v>115</v>
       </c>
       <c r="O35" t="b">
         <v>1</v>
       </c>
       <c r="P35" t="n">
-        <v>50</v>
+        <v>80</v>
       </c>
     </row>
     <row r="36">
@@ -2645,22 +2645,22 @@
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>NC4085-1</t>
+          <t>NC4284</t>
         </is>
       </c>
       <c r="C36" t="inlineStr">
         <is>
-          <t>NC4085-1</t>
+          <t>NC4284_FBA</t>
         </is>
       </c>
       <c r="D36" t="inlineStr">
         <is>
-          <t>B0DDT2TSPK</t>
+          <t>B08Q31XC28</t>
         </is>
       </c>
       <c r="E36" t="inlineStr">
         <is>
-          <t>NC4085-Master</t>
+          <t>NC4059-Master</t>
         </is>
       </c>
       <c r="F36" t="inlineStr">
@@ -2669,34 +2669,34 @@
         </is>
       </c>
       <c r="G36" t="n">
-        <v>15</v>
+        <v>5</v>
       </c>
       <c r="H36" t="n">
-        <v>220</v>
+        <v>80</v>
       </c>
       <c r="I36" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="J36" t="n">
-        <v>69</v>
+        <v>55</v>
       </c>
       <c r="K36" t="n">
-        <v>69</v>
+        <v>55</v>
       </c>
       <c r="L36" t="b">
         <v>0</v>
       </c>
       <c r="M36" t="n">
-        <v>4.57</v>
+        <v>1.86</v>
       </c>
       <c r="N36" t="n">
-        <v>126</v>
+        <v>53</v>
       </c>
       <c r="O36" t="b">
         <v>1</v>
       </c>
       <c r="P36" t="n">
-        <v>40</v>
+        <v>30</v>
       </c>
     </row>
     <row r="37">
@@ -2707,22 +2707,22 @@
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>NC4389</t>
+          <t>NC4059</t>
         </is>
       </c>
       <c r="C37" t="inlineStr">
         <is>
-          <t>NC4389</t>
+          <t>NC4059_FBA</t>
         </is>
       </c>
       <c r="D37" t="inlineStr">
         <is>
-          <t>B0D4DXYK1X</t>
+          <t>B01IACWDOK</t>
         </is>
       </c>
       <c r="E37" t="inlineStr">
         <is>
-          <t>NC4256-Master</t>
+          <t>NC4059-Master</t>
         </is>
       </c>
       <c r="F37" t="inlineStr">
@@ -2731,34 +2731,34 @@
         </is>
       </c>
       <c r="G37" t="n">
-        <v>67</v>
+        <v>20</v>
       </c>
       <c r="H37" t="n">
-        <v>160</v>
+        <v>87</v>
       </c>
       <c r="I37" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="J37" t="n">
-        <v>49</v>
+        <v>41</v>
       </c>
       <c r="K37" t="n">
-        <v>49</v>
+        <v>41</v>
       </c>
       <c r="L37" t="b">
         <v>0</v>
       </c>
       <c r="M37" t="n">
-        <v>6.17</v>
+        <v>2.53</v>
       </c>
       <c r="N37" t="n">
-        <v>180</v>
+        <v>79</v>
       </c>
       <c r="O37" t="b">
         <v>1</v>
       </c>
       <c r="P37" t="n">
-        <v>140</v>
+        <v>40</v>
       </c>
     </row>
     <row r="38">
@@ -2769,22 +2769,22 @@
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>NC4400-A</t>
+          <t>NC4085-1</t>
         </is>
       </c>
       <c r="C38" t="inlineStr">
         <is>
-          <t>NC4400-A</t>
+          <t>NC4085-1</t>
         </is>
       </c>
       <c r="D38" t="inlineStr">
         <is>
-          <t>B0DJSWD9YL</t>
+          <t>B0DDT2TSPK</t>
         </is>
       </c>
       <c r="E38" t="inlineStr">
         <is>
-          <t>NC4400-Master</t>
+          <t>NC4085-Master</t>
         </is>
       </c>
       <c r="F38" t="inlineStr">
@@ -2793,34 +2793,34 @@
         </is>
       </c>
       <c r="G38" t="n">
-        <v>0</v>
+        <v>13</v>
       </c>
       <c r="H38" t="n">
-        <v>140</v>
+        <v>210</v>
       </c>
       <c r="I38" t="n">
-        <v>1</v>
+        <v>8</v>
       </c>
       <c r="J38" t="n">
-        <v>45</v>
+        <v>69</v>
       </c>
       <c r="K38" t="n">
-        <v>0</v>
+        <v>69</v>
       </c>
       <c r="L38" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="M38" t="n">
-        <v>3.19</v>
+        <v>4.46</v>
       </c>
       <c r="N38" t="n">
-        <v>100</v>
+        <v>126</v>
       </c>
       <c r="O38" t="b">
         <v>1</v>
       </c>
       <c r="P38" t="n">
-        <v>60</v>
+        <v>40</v>
       </c>
     </row>
     <row r="39">
@@ -2831,22 +2831,22 @@
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>NC4400-E</t>
+          <t>NC4389</t>
         </is>
       </c>
       <c r="C39" t="inlineStr">
         <is>
-          <t>NC4400-E</t>
+          <t>NC4389</t>
         </is>
       </c>
       <c r="D39" t="inlineStr">
         <is>
-          <t>B0DJSXTMB1</t>
+          <t>B0D4DXYK1X</t>
         </is>
       </c>
       <c r="E39" t="inlineStr">
         <is>
-          <t>NC4400-Master</t>
+          <t>NC4256-Master</t>
         </is>
       </c>
       <c r="F39" t="inlineStr">
@@ -2855,13 +2855,13 @@
         </is>
       </c>
       <c r="G39" t="n">
+        <v>65</v>
+      </c>
+      <c r="H39" t="n">
+        <v>160</v>
+      </c>
+      <c r="I39" t="n">
         <v>6</v>
-      </c>
-      <c r="H39" t="n">
-        <v>100</v>
-      </c>
-      <c r="I39" t="n">
-        <v>0</v>
       </c>
       <c r="J39" t="n">
         <v>48</v>
@@ -2873,16 +2873,16 @@
         <v>0</v>
       </c>
       <c r="M39" t="n">
-        <v>2.04</v>
+        <v>6.16</v>
       </c>
       <c r="N39" t="n">
-        <v>75</v>
+        <v>180</v>
       </c>
       <c r="O39" t="b">
         <v>1</v>
       </c>
       <c r="P39" t="n">
-        <v>20</v>
+        <v>140</v>
       </c>
     </row>
     <row r="40">
@@ -2893,17 +2893,17 @@
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>NC4400-H</t>
+          <t>NC4400-A</t>
         </is>
       </c>
       <c r="C40" t="inlineStr">
         <is>
-          <t>NC4400-H</t>
+          <t>NC4400-A</t>
         </is>
       </c>
       <c r="D40" t="inlineStr">
         <is>
-          <t>B0DJSXXKS8</t>
+          <t>B0DJSWD9YL</t>
         </is>
       </c>
       <c r="E40" t="inlineStr">
@@ -2917,34 +2917,34 @@
         </is>
       </c>
       <c r="G40" t="n">
-        <v>43</v>
+        <v>0</v>
       </c>
       <c r="H40" t="n">
-        <v>0</v>
+        <v>140</v>
       </c>
       <c r="I40" t="n">
         <v>2</v>
       </c>
       <c r="J40" t="n">
-        <v>15</v>
+        <v>44</v>
       </c>
       <c r="K40" t="n">
-        <v>15</v>
+        <v>0</v>
       </c>
       <c r="L40" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="M40" t="n">
-        <v>0.79</v>
+        <v>3.13</v>
       </c>
       <c r="N40" t="n">
-        <v>34</v>
+        <v>100</v>
       </c>
       <c r="O40" t="b">
         <v>1</v>
       </c>
       <c r="P40" t="n">
-        <v>10</v>
+        <v>50</v>
       </c>
     </row>
     <row r="41">
@@ -2955,17 +2955,17 @@
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>NC4400-L1</t>
+          <t>NC4400-E</t>
         </is>
       </c>
       <c r="C41" t="inlineStr">
         <is>
-          <t>NC4400-L1</t>
+          <t>NC4400-E</t>
         </is>
       </c>
       <c r="D41" t="inlineStr">
         <is>
-          <t>B0FJ1Z3LVM</t>
+          <t>B0DJSXTMB1</t>
         </is>
       </c>
       <c r="E41" t="inlineStr">
@@ -2979,28 +2979,28 @@
         </is>
       </c>
       <c r="G41" t="n">
-        <v>17</v>
+        <v>5</v>
       </c>
       <c r="H41" t="n">
-        <v>40</v>
+        <v>100</v>
       </c>
       <c r="I41" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J41" t="n">
-        <v>2</v>
+        <v>48</v>
       </c>
       <c r="K41" t="n">
-        <v>2</v>
+        <v>48</v>
       </c>
       <c r="L41" t="b">
         <v>0</v>
       </c>
       <c r="M41" t="n">
-        <v>1.27</v>
+        <v>2.07</v>
       </c>
       <c r="N41" t="n">
-        <v>44</v>
+        <v>75</v>
       </c>
       <c r="O41" t="b">
         <v>1</v>
@@ -3017,57 +3017,181 @@
       </c>
       <c r="B42" t="inlineStr">
         <is>
+          <t>NC4400-H</t>
+        </is>
+      </c>
+      <c r="C42" t="inlineStr">
+        <is>
+          <t>NC4400-H</t>
+        </is>
+      </c>
+      <c r="D42" t="inlineStr">
+        <is>
+          <t>B0DJSXXKS8</t>
+        </is>
+      </c>
+      <c r="E42" t="inlineStr">
+        <is>
+          <t>NC4400-Master</t>
+        </is>
+      </c>
+      <c r="F42" t="inlineStr">
+        <is>
+          <t>NC</t>
+        </is>
+      </c>
+      <c r="G42" t="n">
+        <v>43</v>
+      </c>
+      <c r="H42" t="n">
+        <v>0</v>
+      </c>
+      <c r="I42" t="n">
+        <v>1</v>
+      </c>
+      <c r="J42" t="n">
+        <v>15</v>
+      </c>
+      <c r="K42" t="n">
+        <v>15</v>
+      </c>
+      <c r="L42" t="b">
+        <v>0</v>
+      </c>
+      <c r="M42" t="n">
+        <v>0.78</v>
+      </c>
+      <c r="N42" t="n">
+        <v>34</v>
+      </c>
+      <c r="O42" t="b">
+        <v>1</v>
+      </c>
+      <c r="P42" t="n">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" t="inlineStr">
+        <is>
+          <t>NC CHOKERS</t>
+        </is>
+      </c>
+      <c r="B43" t="inlineStr">
+        <is>
+          <t>NC4400-L1</t>
+        </is>
+      </c>
+      <c r="C43" t="inlineStr">
+        <is>
+          <t>NC4400-L1</t>
+        </is>
+      </c>
+      <c r="D43" t="inlineStr">
+        <is>
+          <t>B0FJ1Z3LVM</t>
+        </is>
+      </c>
+      <c r="E43" t="inlineStr">
+        <is>
+          <t>NC4400-Master</t>
+        </is>
+      </c>
+      <c r="F43" t="inlineStr">
+        <is>
+          <t>NC</t>
+        </is>
+      </c>
+      <c r="G43" t="n">
+        <v>17</v>
+      </c>
+      <c r="H43" t="n">
+        <v>40</v>
+      </c>
+      <c r="I43" t="n">
+        <v>0</v>
+      </c>
+      <c r="J43" t="n">
+        <v>2</v>
+      </c>
+      <c r="K43" t="n">
+        <v>2</v>
+      </c>
+      <c r="L43" t="b">
+        <v>0</v>
+      </c>
+      <c r="M43" t="n">
+        <v>1.26</v>
+      </c>
+      <c r="N43" t="n">
+        <v>44</v>
+      </c>
+      <c r="O43" t="b">
+        <v>1</v>
+      </c>
+      <c r="P43" t="n">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" t="inlineStr">
+        <is>
+          <t>NC CHOKERS</t>
+        </is>
+      </c>
+      <c r="B44" t="inlineStr">
+        <is>
           <t>NC4400-S</t>
         </is>
       </c>
-      <c r="C42" t="inlineStr">
+      <c r="C44" t="inlineStr">
         <is>
           <t>NC4400-S</t>
         </is>
       </c>
-      <c r="D42" t="inlineStr">
+      <c r="D44" t="inlineStr">
         <is>
           <t>B0DJSX3BG2</t>
         </is>
       </c>
-      <c r="E42" t="inlineStr">
+      <c r="E44" t="inlineStr">
         <is>
           <t>NC4400-Master</t>
         </is>
       </c>
-      <c r="F42" t="inlineStr">
+      <c r="F44" t="inlineStr">
         <is>
           <t>NC</t>
         </is>
       </c>
-      <c r="G42" t="n">
-        <v>42</v>
-      </c>
-      <c r="H42" t="n">
-        <v>0</v>
-      </c>
-      <c r="I42" t="n">
-        <v>1</v>
-      </c>
-      <c r="J42" t="n">
-        <v>0</v>
-      </c>
-      <c r="K42" t="n">
-        <v>38.5</v>
-      </c>
-      <c r="L42" t="b">
-        <v>0</v>
-      </c>
-      <c r="M42" t="n">
-        <v>1.09</v>
-      </c>
-      <c r="N42" t="n">
+      <c r="G44" t="n">
+        <v>44</v>
+      </c>
+      <c r="H44" t="n">
+        <v>0</v>
+      </c>
+      <c r="I44" t="n">
+        <v>0</v>
+      </c>
+      <c r="J44" t="n">
+        <v>1</v>
+      </c>
+      <c r="K44" t="n">
+        <v>1</v>
+      </c>
+      <c r="L44" t="b">
+        <v>0</v>
+      </c>
+      <c r="M44" t="n">
+        <v>1.1</v>
+      </c>
+      <c r="N44" t="n">
         <v>35</v>
       </c>
-      <c r="O42" t="b">
-        <v>1</v>
-      </c>
-      <c r="P42" t="n">
+      <c r="O44" t="b">
+        <v>1</v>
+      </c>
+      <c r="P44" t="n">
         <v>30</v>
       </c>
     </row>
@@ -3117,7 +3241,7 @@
         <v>7</v>
       </c>
       <c r="C2" t="n">
-        <v>120</v>
+        <v>110</v>
       </c>
     </row>
     <row r="3">
@@ -3140,10 +3264,10 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>7</v>
+        <v>9</v>
       </c>
       <c r="C4" t="n">
-        <v>340</v>
+        <v>350</v>
       </c>
     </row>
     <row r="5">
@@ -3156,7 +3280,7 @@
         <v>18</v>
       </c>
       <c r="C5" t="n">
-        <v>1240</v>
+        <v>1120</v>
       </c>
     </row>
     <row r="6">
@@ -3166,10 +3290,10 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>41</v>
+        <v>43</v>
       </c>
       <c r="C6" t="n">
-        <v>2090</v>
+        <v>1970</v>
       </c>
     </row>
   </sheetData>

</xml_diff>